<commit_message>
feat: update crawl 5/9
</commit_message>
<xml_diff>
--- a/outputs/vps-crawl-planner-20260823/vps_crawl_sampling_master.xlsx
+++ b/outputs/vps-crawl-planner-20260823/vps_crawl_sampling_master.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" r:id="Re70581b677b843ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VPS_CRAWL_PLAN" sheetId="2" r:id="R5e3b034bc8774328"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRAWL_LOG" sheetId="3" r:id="R9fb478aa3479445f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOCAL_REFERENCE" sheetId="4" r:id="R5a3f60c5ee494cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLOT_RULES" sheetId="5" r:id="Rd5123d728d2d4dc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" r:id="Rd11f3bcbdd7c495d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" r:id="R90aa0cd8e47647d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VPS_CRAWL_PLAN" sheetId="2" r:id="R992edd0fa285454f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRAWL_LOG" sheetId="3" r:id="R7c3d6f2c7e2d4eb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOCAL_REFERENCE" sheetId="4" r:id="R552904b42fdf44c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLOT_RULES" sheetId="5" r:id="R200edea7866e4799"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" r:id="R2cb35b2e34d74e77"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,12 +18,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0"/>
     <x:numFmt numFmtId="203" formatCode="dd/mm/yyyy hh:mm"/>
     <x:numFmt numFmtId="204" formatCode="0.00"/>
+    <x:numFmt numFmtId="205" formatCode="dd/mm/yyyy hh:mm:ss"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -208,7 +209,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="71">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -326,6 +327,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -870,7 +872,7 @@
       </x:c>
       <x:c r="B12" s="28" t="n">
         <x:f>COUNTIF('CRAWL_LOG'!$B$4:$B$102,"Hoàn thành")+COUNTIF('CRAWL_LOG'!$B$4:$B$102,"Hoàn thành có lỗi")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -879,7 +881,7 @@
       </x:c>
       <x:c r="B13" s="29" t="n">
         <x:f>COUNTIF('CRAWL_LOG'!$B$4:$B$102,"Chưa chạy")</x:f>
-        <x:v>87</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1762,7 +1764,7 @@
       </x:c>
       <x:c r="N16" s="36" t="str">
         <x:f>'CRAWL_LOG'!B16</x:f>
-        <x:v>Chưa chạy</x:v>
+        <x:v>Hoàn thành có lỗi</x:v>
       </x:c>
       <x:c r="O16" s="36" t="str">
         <x:v>Supplementary panel</x:v>
@@ -6252,7 +6254,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2600ce08d8ec436f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3984f84f59b4703"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7082,29 +7084,53 @@
         <x:v>46270</x:v>
       </x:c>
       <x:c r="B16" s="36" t="str">
-        <x:v>Chưa chạy</x:v>
-      </x:c>
-      <x:c r="C16" s="36"/>
-      <x:c r="D16" s="44"/>
-      <x:c r="E16" s="44"/>
-      <x:c r="F16" s="46" t="str">
-        <x:f>IF(OR(D16="",E16=""),"",24*(E16-D16))</x:f>
-      </x:c>
-      <x:c r="G16" s="48"/>
-      <x:c r="H16" s="48"/>
-      <x:c r="I16" s="48"/>
-      <x:c r="J16" s="48"/>
-      <x:c r="K16" s="48"/>
-      <x:c r="L16" s="48"/>
-      <x:c r="M16" s="48"/>
-      <x:c r="N16" s="48"/>
+        <x:v>Hoàn thành có lỗi</x:v>
+      </x:c>
+      <x:c r="C16" s="36" t="str">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D16" s="71" t="n">
+        <x:v>46270.0231712963</x:v>
+      </x:c>
+      <x:c r="E16" s="44" t="n">
+        <x:v>46270.93908564815</x:v>
+      </x:c>
+      <x:c r="F16" s="46" t="n">
+        <x:v>21.981944444356486</x:v>
+      </x:c>
+      <x:c r="G16" s="48" t="n">
+        <x:v>1770</x:v>
+      </x:c>
+      <x:c r="H16" s="48" t="n">
+        <x:v>1770</x:v>
+      </x:c>
+      <x:c r="I16" s="48" t="n">
+        <x:v>1583</x:v>
+      </x:c>
+      <x:c r="J16" s="48" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K16" s="48" t="n">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="L16" s="48" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="M16" s="48" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N16" s="48" t="n">
+        <x:v>14706</x:v>
+      </x:c>
       <x:c r="O16" s="48" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="P16" s="36" t="str">
         <x:v>vps</x:v>
       </x:c>
-      <x:c r="Q16" s="36"/>
+      <x:c r="Q16" s="36" t="str">
+        <x:v>Run ID 15; deploy https://hotel.projecthub.io.vn/; artifact không lưu; scraper_version 2.3.0; terminal API status completed; items pagination 1770; saved_options_count 14706.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="40" t="n">
@@ -9617,7 +9643,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb38d7f1a24da4aa6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R978870dbcdca4fd2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14751,7 +14777,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf1eadf343c849a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06f786ee14f84fcb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14964,7 +14990,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd42d49338ec24d72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re24dce093d5b4ff8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15111,7 +15137,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ab18cf4da97409e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b46bf4fab604294"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update crawl 10/9
</commit_message>
<xml_diff>
--- a/outputs/vps-crawl-planner-20260823/vps_crawl_sampling_master.xlsx
+++ b/outputs/vps-crawl-planner-20260823/vps_crawl_sampling_master.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" r:id="R334190919a9b4191"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VPS_CRAWL_PLAN" sheetId="2" r:id="R8b0b6d2b1c35439c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRAWL_LOG" sheetId="3" r:id="Readaa929ae354ffd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOCAL_REFERENCE" sheetId="4" r:id="R567bb33dc7b54542"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLOT_RULES" sheetId="5" r:id="R50ea720fbca14fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" r:id="R1d1f87b967ad48bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" r:id="Rf631b05d1b5941bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VPS_CRAWL_PLAN" sheetId="2" r:id="Rf9b9201294154f65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRAWL_LOG" sheetId="3" r:id="R3f7f49e745e0482b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOCAL_REFERENCE" sheetId="4" r:id="R51ee3179bd574fd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLOT_RULES" sheetId="5" r:id="Rbe749ec118974481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" r:id="Re45acd104b3f406d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -985,7 +985,7 @@
       </x:c>
       <x:c r="B12" s="74" t="n">
         <x:f>COUNTIF('CRAWL_LOG'!$B$4:$B$102,"Hoàn thành")+COUNTIF('CRAWL_LOG'!$B$4:$B$102,"Hoàn thành có lỗi")</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -996,7 +996,7 @@
       </x:c>
       <x:c r="B13" s="75" t="n">
         <x:f>COUNTIF('CRAWL_LOG'!$B$4:$B$102,"Chưa chạy")</x:f>
-        <x:v>83</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2145,7 +2145,7 @@
       </x:c>
       <x:c r="N20" s="36" t="str">
         <x:f>'CRAWL_LOG'!B20</x:f>
-        <x:v>Chưa chạy</x:v>
+        <x:v>Hoàn thành có lỗi</x:v>
       </x:c>
       <x:c r="O20" s="36" t="inlineStr">
         <x:is>
@@ -7085,7 +7085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d4e4f9dde034673"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc447ae44a6c34a0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8152,34 +8152,54 @@
       <x:c r="A20" s="76" t="n">
         <x:v>46274</x:v>
       </x:c>
-      <x:c r="B20" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chưa chạy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C20" s="36" t="n"/>
-      <x:c r="D20" s="81" t="n"/>
-      <x:c r="E20" s="81" t="n"/>
-      <x:c r="F20" s="82" t="str">
-        <x:f>IF(OR(D20="",E20=""),"",24*(E20-D20))</x:f>
-      </x:c>
-      <x:c r="G20" s="83" t="n"/>
-      <x:c r="H20" s="83" t="n"/>
-      <x:c r="I20" s="83" t="n"/>
-      <x:c r="J20" s="83" t="n"/>
-      <x:c r="K20" s="83" t="n"/>
-      <x:c r="L20" s="83" t="n"/>
-      <x:c r="M20" s="83" t="n"/>
-      <x:c r="N20" s="83" t="n"/>
+      <x:c r="B20" s="36" t="str">
+        <x:v>Hoàn thành có lỗi</x:v>
+      </x:c>
+      <x:c r="C20" s="36" t="str">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D20" s="81" t="n">
+        <x:v>46274.02339120371</x:v>
+      </x:c>
+      <x:c r="E20" s="81" t="n">
+        <x:v>46274.92560185185</x:v>
+      </x:c>
+      <x:c r="F20" s="82" t="n">
+        <x:v>21.653055555555557</x:v>
+      </x:c>
+      <x:c r="G20" s="83" t="n">
+        <x:v>1770</x:v>
+      </x:c>
+      <x:c r="H20" s="83" t="n">
+        <x:v>1770</x:v>
+      </x:c>
+      <x:c r="I20" s="83" t="n">
+        <x:v>1574</x:v>
+      </x:c>
+      <x:c r="J20" s="83" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K20" s="83" t="n">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="L20" s="83" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="M20" s="83" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N20" s="83" t="n">
+        <x:v>15038</x:v>
+      </x:c>
       <x:c r="O20" s="83" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="P20" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">vps</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q20" s="36" t="n"/>
+      <x:c r="P20" s="36" t="str">
+        <x:v>vps</x:v>
+      </x:c>
+      <x:c r="Q20" s="36" t="str">
+        <x:v>Run ID 19; deploy https://hotel.projecthub.io.vn/; artifact không lưu; scraper_version 2.3.0; terminal API status completed; items pagination 1770; saved_options_count 15038.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="79" t="n">
@@ -10904,7 +10924,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c48ecdc5a3449b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51a68b3337454f99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16578,7 +16598,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabdf69b747974a95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d134c63474146dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16868,7 +16888,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9898746c6ccb48d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R113122d8bbc647bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17058,7 +17078,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08c2913ac9114aaf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d284580d01847c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>